<commit_message>
Implement parallel execution with JUnit 5 Platform and keep TestRunner.java unchanged
</commit_message>
<xml_diff>
--- a/testdatafolder/HomeLoan_15Lac_9_5_1Year.xlsx
+++ b/testdatafolder/HomeLoan_15Lac_9_5_1Year.xlsx
@@ -12,16 +12,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="30">
   <si>
     <t>Year</t>
   </si>
   <si>
     <t>Principal
 (A)</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Interest
@@ -153,17 +150,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="7.921875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="9.921875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="8.921875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="11.4140625" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="12.55078125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="11.4140625" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="12.55078125" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="7.19921875" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="15.37890625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="15.37890625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -180,16 +175,10 @@
         <v>3</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s" s="0">
         <v>5</v>
-      </c>
-      <c r="H1" t="s" s="0">
-        <v>6</v>
       </c>
     </row>
     <row r="2">
@@ -209,12 +198,12 @@
         <v>515851.0</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" t="n" s="1">
         <v>119650.0</v>
@@ -229,12 +218,12 @@
         <v>1380350.0</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" t="n" s="1">
         <v>120597.0</v>
@@ -249,12 +238,12 @@
         <v>1259752.0</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" t="n" s="1">
         <v>121552.0</v>
@@ -269,12 +258,12 @@
         <v>1138200.0</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="n" s="1">
         <v>122515.0</v>
@@ -289,12 +278,12 @@
         <v>1015685.0</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" t="n" s="1">
         <v>123484.0</v>
@@ -309,12 +298,12 @@
         <v>892201.0</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" t="n" s="1">
         <v>124462.0</v>
@@ -329,12 +318,12 @@
         <v>767739.0</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B9" t="n" s="1">
         <v>125447.0</v>
@@ -349,12 +338,12 @@
         <v>642292.0</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10" t="n" s="1">
         <v>126440.0</v>
@@ -369,12 +358,12 @@
         <v>515851.0</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B11" t="n" s="1">
         <v>119650.0</v>
@@ -389,12 +378,12 @@
         <v>1380350.0</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" t="n" s="1">
         <v>120597.0</v>
@@ -409,12 +398,12 @@
         <v>1259752.0</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="n" s="1">
         <v>121552.0</v>
@@ -429,12 +418,12 @@
         <v>1138200.0</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="n" s="1">
         <v>122515.0</v>
@@ -449,12 +438,12 @@
         <v>1015685.0</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" t="n" s="1">
         <v>123484.0</v>
@@ -469,12 +458,12 @@
         <v>892201.0</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" t="n" s="1">
         <v>124462.0</v>
@@ -489,12 +478,12 @@
         <v>767739.0</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17" t="n" s="1">
         <v>125447.0</v>
@@ -509,12 +498,12 @@
         <v>642292.0</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B18" t="n" s="1">
         <v>126440.0</v>
@@ -529,7 +518,7 @@
         <v>515851.0</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -549,12 +538,12 @@
         <v>0.0</v>
       </c>
       <c r="F19" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B20" t="n" s="1">
         <v>127441.0</v>
@@ -569,12 +558,12 @@
         <v>388410.0</v>
       </c>
       <c r="F20" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" t="n" s="1">
         <v>128450.0</v>
@@ -589,12 +578,12 @@
         <v>259959.0</v>
       </c>
       <c r="F21" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" t="n" s="1">
         <v>129467.0</v>
@@ -609,12 +598,12 @@
         <v>130492.0</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" t="n" s="1">
         <v>130492.0</v>
@@ -629,12 +618,12 @@
         <v>0.0</v>
       </c>
       <c r="F23" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" t="n" s="1">
         <v>127441.0</v>
@@ -649,12 +638,12 @@
         <v>388410.0</v>
       </c>
       <c r="F24" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25" t="n" s="1">
         <v>128450.0</v>
@@ -669,12 +658,12 @@
         <v>259959.0</v>
       </c>
       <c r="F25" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B26" t="n" s="1">
         <v>129467.0</v>
@@ -689,12 +678,12 @@
         <v>130492.0</v>
       </c>
       <c r="F26" t="s" s="0">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B27" t="n" s="1">
         <v>130492.0</v>
@@ -709,7 +698,7 @@
         <v>0.0</v>
       </c>
       <c r="F27" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>